<commit_message>
R1-R3 TST rescue: backfill 30d LSR/OI + CASE_TST DAILY merge + GOM analysis
R1: collect_daily_metrics --symbols TSTUSDT --days-back 30 (VPS, errors=0)
R2: 5 metrics x 30 dates verified; MISSING-PERMANENT < 07-10/07-11
R3: Merge pos_r/acc_r/gLSR/taker_lsr + div_raw/avg3 vào CASE_TST DAILY (29 rows)
ANALYSIS: TST GOM = 0/545 fire (100% ABSTAIN). Blocker cứng: A2 (avg5 gLSR 1.54-2.37 >> 1.1)
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_TST.xlsx
+++ b/docs/case_files/CASE_TST.xlsx
@@ -65180,7 +65180,9 @@
       <c r="V506" s="14" t="n">
         <v>1.4712</v>
       </c>
-      <c r="W506" s="14" t="inlineStr"/>
+      <c r="W506" s="14" t="n">
+        <v>1.4712</v>
+      </c>
       <c r="X506" s="14" t="inlineStr"/>
       <c r="Y506" s="14" t="inlineStr"/>
       <c r="Z506" s="14" t="inlineStr"/>
@@ -65328,7 +65330,9 @@
       <c r="V507" s="14" t="n">
         <v>1.4306</v>
       </c>
-      <c r="W507" s="14" t="inlineStr"/>
+      <c r="W507" s="14" t="n">
+        <v>1.4509</v>
+      </c>
       <c r="X507" s="14" t="inlineStr"/>
       <c r="Y507" s="14" t="inlineStr"/>
       <c r="Z507" s="14" t="inlineStr"/>
@@ -65477,7 +65481,7 @@
         <v>1.3674</v>
       </c>
       <c r="W508" s="14" t="n">
-        <v>1.4207</v>
+        <v>1.4231</v>
       </c>
       <c r="X508" s="14" t="inlineStr"/>
       <c r="Y508" s="14" t="inlineStr"/>
@@ -65627,7 +65631,7 @@
         <v>1.3083</v>
       </c>
       <c r="W509" s="14" t="n">
-        <v>1.3649</v>
+        <v>1.3688</v>
       </c>
       <c r="X509" s="14" t="inlineStr"/>
       <c r="Y509" s="14" t="n">
@@ -65781,7 +65785,7 @@
         <v>1.2578</v>
       </c>
       <c r="W510" s="14" t="n">
-        <v>1.3088</v>
+        <v>1.3112</v>
       </c>
       <c r="X510" s="14" t="inlineStr"/>
       <c r="Y510" s="14" t="n">
@@ -65935,7 +65939,7 @@
         <v>1.205</v>
       </c>
       <c r="W511" s="14" t="n">
-        <v>1.255</v>
+        <v>1.257</v>
       </c>
       <c r="X511" s="14" t="n">
         <v>1.5433</v>
@@ -66091,7 +66095,7 @@
         <v>1.2705</v>
       </c>
       <c r="W512" s="14" t="n">
-        <v>1.2449</v>
+        <v>1.2444</v>
       </c>
       <c r="X512" s="14" t="n">
         <v>1.5995</v>
@@ -66247,7 +66251,7 @@
         <v>1.293</v>
       </c>
       <c r="W513" s="14" t="n">
-        <v>1.2581</v>
+        <v>1.2562</v>
       </c>
       <c r="X513" s="14" t="n">
         <v>1.4748</v>
@@ -66403,7 +66407,7 @@
         <v>1.0904</v>
       </c>
       <c r="W514" s="14" t="n">
-        <v>1.2078</v>
+        <v>1.218</v>
       </c>
       <c r="X514" s="14" t="n">
         <v>1.4486</v>
@@ -66559,7 +66563,7 @@
         <v>1.0161</v>
       </c>
       <c r="W515" s="14" t="n">
-        <v>1.1196</v>
+        <v>1.1332</v>
       </c>
       <c r="X515" s="14" t="n">
         <v>1.4738</v>
@@ -66715,7 +66719,7 @@
         <v>1.2229</v>
       </c>
       <c r="W516" s="14" t="n">
-        <v>1.0927</v>
+        <v>1.1098</v>
       </c>
       <c r="X516" s="14" t="n">
         <v>0.7329</v>
@@ -66871,7 +66875,7 @@
         <v>0.9175</v>
       </c>
       <c r="W517" s="14" t="n">
-        <v>1.0503</v>
+        <v>1.0522</v>
       </c>
       <c r="X517" s="14" t="n">
         <v>0.6244</v>
@@ -67173,7 +67177,9 @@
       <c r="AA519" s="14" t="inlineStr"/>
       <c r="AB519" s="14" t="inlineStr"/>
       <c r="AC519" s="14" t="inlineStr"/>
-      <c r="AD519" s="14" t="inlineStr"/>
+      <c r="AD519" s="14" t="n">
+        <v>0.7729</v>
+      </c>
       <c r="AE519" s="14" t="inlineStr"/>
       <c r="AF519" s="14" t="inlineStr"/>
       <c r="AG519" s="14" t="inlineStr"/>
@@ -67307,15 +67313,27 @@
       <c r="U520" s="14" t="n">
         <v>0.98</v>
       </c>
-      <c r="V520" s="14" t="inlineStr"/>
-      <c r="W520" s="14" t="inlineStr"/>
+      <c r="V520" s="14" t="n">
+        <v>0.7079</v>
+      </c>
+      <c r="W520" s="14" t="n">
+        <v>0.7079</v>
+      </c>
       <c r="X520" s="14" t="inlineStr"/>
       <c r="Y520" s="14" t="inlineStr"/>
       <c r="Z520" s="14" t="inlineStr"/>
-      <c r="AA520" s="14" t="inlineStr"/>
-      <c r="AB520" s="14" t="inlineStr"/>
-      <c r="AC520" s="14" t="inlineStr"/>
-      <c r="AD520" s="14" t="inlineStr"/>
+      <c r="AA520" s="14" t="n">
+        <v>1.3031</v>
+      </c>
+      <c r="AB520" s="14" t="n">
+        <v>1.8409</v>
+      </c>
+      <c r="AC520" s="14" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="AD520" s="14" t="n">
+        <v>0.9893</v>
+      </c>
       <c r="AE520" s="14" t="inlineStr"/>
       <c r="AF520" s="14" t="inlineStr"/>
       <c r="AG520" s="14" t="inlineStr"/>
@@ -67449,15 +67467,27 @@
       <c r="U521" s="14" t="n">
         <v>2.47</v>
       </c>
-      <c r="V521" s="14" t="inlineStr"/>
-      <c r="W521" s="14" t="inlineStr"/>
+      <c r="V521" s="14" t="n">
+        <v>0.7133</v>
+      </c>
+      <c r="W521" s="14" t="n">
+        <v>0.7106</v>
+      </c>
       <c r="X521" s="14" t="inlineStr"/>
       <c r="Y521" s="14" t="inlineStr"/>
       <c r="Z521" s="14" t="inlineStr"/>
-      <c r="AA521" s="14" t="inlineStr"/>
-      <c r="AB521" s="14" t="inlineStr"/>
-      <c r="AC521" s="14" t="inlineStr"/>
-      <c r="AD521" s="14" t="inlineStr"/>
+      <c r="AA521" s="14" t="n">
+        <v>1.3971</v>
+      </c>
+      <c r="AB521" s="14" t="n">
+        <v>1.9586</v>
+      </c>
+      <c r="AC521" s="14" t="n">
+        <v>1.666</v>
+      </c>
+      <c r="AD521" s="14" t="n">
+        <v>1.04</v>
+      </c>
       <c r="AE521" s="14" t="inlineStr"/>
       <c r="AF521" s="14" t="inlineStr"/>
       <c r="AG521" s="14" t="inlineStr"/>
@@ -67591,15 +67621,27 @@
       <c r="U522" s="14" t="n">
         <v>1.44</v>
       </c>
-      <c r="V522" s="14" t="inlineStr"/>
-      <c r="W522" s="14" t="inlineStr"/>
+      <c r="V522" s="14" t="n">
+        <v>0.8318</v>
+      </c>
+      <c r="W522" s="14" t="n">
+        <v>0.751</v>
+      </c>
       <c r="X522" s="14" t="inlineStr"/>
       <c r="Y522" s="14" t="inlineStr"/>
       <c r="Z522" s="14" t="inlineStr"/>
-      <c r="AA522" s="14" t="inlineStr"/>
-      <c r="AB522" s="14" t="inlineStr"/>
-      <c r="AC522" s="14" t="inlineStr"/>
-      <c r="AD522" s="14" t="inlineStr"/>
+      <c r="AA522" s="14" t="n">
+        <v>1.5632</v>
+      </c>
+      <c r="AB522" s="14" t="n">
+        <v>1.8794</v>
+      </c>
+      <c r="AC522" s="14" t="n">
+        <v>1.6247</v>
+      </c>
+      <c r="AD522" s="14" t="n">
+        <v>1.0049</v>
+      </c>
       <c r="AE522" s="14" t="inlineStr"/>
       <c r="AF522" s="14" t="inlineStr"/>
       <c r="AG522" s="14" t="inlineStr"/>
@@ -67733,15 +67775,27 @@
       <c r="U523" s="14" t="n">
         <v>1.09</v>
       </c>
-      <c r="V523" s="14" t="inlineStr"/>
-      <c r="W523" s="14" t="inlineStr"/>
+      <c r="V523" s="14" t="n">
+        <v>0.8389</v>
+      </c>
+      <c r="W523" s="14" t="n">
+        <v>0.7947</v>
+      </c>
       <c r="X523" s="14" t="inlineStr"/>
       <c r="Y523" s="14" t="inlineStr"/>
       <c r="Z523" s="14" t="inlineStr"/>
-      <c r="AA523" s="14" t="inlineStr"/>
-      <c r="AB523" s="14" t="inlineStr"/>
-      <c r="AC523" s="14" t="inlineStr"/>
-      <c r="AD523" s="14" t="inlineStr"/>
+      <c r="AA523" s="14" t="n">
+        <v>1.496</v>
+      </c>
+      <c r="AB523" s="14" t="n">
+        <v>1.7832</v>
+      </c>
+      <c r="AC523" s="14" t="n">
+        <v>1.5381</v>
+      </c>
+      <c r="AD523" s="14" t="n">
+        <v>0.985</v>
+      </c>
       <c r="AE523" s="14" t="inlineStr"/>
       <c r="AF523" s="14" t="inlineStr"/>
       <c r="AG523" s="14" t="inlineStr"/>
@@ -67875,15 +67929,27 @@
       <c r="U524" s="14" t="n">
         <v>0.51</v>
       </c>
-      <c r="V524" s="14" t="inlineStr"/>
-      <c r="W524" s="14" t="inlineStr"/>
+      <c r="V524" s="14" t="n">
+        <v>0.7935</v>
+      </c>
+      <c r="W524" s="14" t="n">
+        <v>0.8214</v>
+      </c>
       <c r="X524" s="14" t="inlineStr"/>
       <c r="Y524" s="14" t="inlineStr"/>
       <c r="Z524" s="14" t="inlineStr"/>
-      <c r="AA524" s="14" t="inlineStr"/>
-      <c r="AB524" s="14" t="inlineStr"/>
-      <c r="AC524" s="14" t="inlineStr"/>
-      <c r="AD524" s="14" t="inlineStr"/>
+      <c r="AA524" s="14" t="n">
+        <v>1.4506</v>
+      </c>
+      <c r="AB524" s="14" t="n">
+        <v>1.8281</v>
+      </c>
+      <c r="AC524" s="14" t="n">
+        <v>1.7412</v>
+      </c>
+      <c r="AD524" s="14" t="n">
+        <v>0.9588</v>
+      </c>
       <c r="AE524" s="14" t="inlineStr"/>
       <c r="AF524" s="14" t="inlineStr"/>
       <c r="AG524" s="14" t="inlineStr"/>
@@ -68017,15 +68083,27 @@
       <c r="U525" s="14" t="n">
         <v>0.43</v>
       </c>
-      <c r="V525" s="14" t="inlineStr"/>
-      <c r="W525" s="14" t="inlineStr"/>
+      <c r="V525" s="14" t="n">
+        <v>0.7251</v>
+      </c>
+      <c r="W525" s="14" t="n">
+        <v>0.7858000000000001</v>
+      </c>
       <c r="X525" s="14" t="inlineStr"/>
       <c r="Y525" s="14" t="inlineStr"/>
       <c r="Z525" s="14" t="inlineStr"/>
-      <c r="AA525" s="14" t="inlineStr"/>
-      <c r="AB525" s="14" t="inlineStr"/>
-      <c r="AC525" s="14" t="inlineStr"/>
-      <c r="AD525" s="14" t="inlineStr"/>
+      <c r="AA525" s="14" t="n">
+        <v>1.4479</v>
+      </c>
+      <c r="AB525" s="14" t="n">
+        <v>1.9967</v>
+      </c>
+      <c r="AC525" s="14" t="n">
+        <v>1.8629</v>
+      </c>
+      <c r="AD525" s="14" t="n">
+        <v>0.7798</v>
+      </c>
       <c r="AE525" s="14" t="inlineStr"/>
       <c r="AF525" s="14" t="inlineStr"/>
       <c r="AG525" s="14" t="inlineStr"/>
@@ -68161,15 +68239,27 @@
       <c r="U526" s="14" t="n">
         <v>0.37</v>
       </c>
-      <c r="V526" s="14" t="inlineStr"/>
-      <c r="W526" s="14" t="inlineStr"/>
+      <c r="V526" s="14" t="n">
+        <v>0.7698</v>
+      </c>
+      <c r="W526" s="14" t="n">
+        <v>0.7628</v>
+      </c>
       <c r="X526" s="14" t="inlineStr"/>
       <c r="Y526" s="14" t="inlineStr"/>
       <c r="Z526" s="14" t="inlineStr"/>
-      <c r="AA526" s="14" t="inlineStr"/>
-      <c r="AB526" s="14" t="inlineStr"/>
-      <c r="AC526" s="14" t="inlineStr"/>
-      <c r="AD526" s="14" t="inlineStr"/>
+      <c r="AA526" s="14" t="n">
+        <v>1.5686</v>
+      </c>
+      <c r="AB526" s="14" t="n">
+        <v>2.0377</v>
+      </c>
+      <c r="AC526" s="14" t="n">
+        <v>1.9231</v>
+      </c>
+      <c r="AD526" s="14" t="n">
+        <v>0.9174</v>
+      </c>
       <c r="AE526" s="14" t="inlineStr"/>
       <c r="AF526" s="14" t="inlineStr"/>
       <c r="AG526" s="14" t="inlineStr"/>
@@ -68305,15 +68395,27 @@
       <c r="U527" s="14" t="n">
         <v>0.3</v>
       </c>
-      <c r="V527" s="14" t="inlineStr"/>
-      <c r="W527" s="14" t="inlineStr"/>
+      <c r="V527" s="14" t="n">
+        <v>0.8772</v>
+      </c>
+      <c r="W527" s="14" t="n">
+        <v>0.7907</v>
+      </c>
       <c r="X527" s="14" t="inlineStr"/>
       <c r="Y527" s="14" t="inlineStr"/>
       <c r="Z527" s="14" t="inlineStr"/>
-      <c r="AA527" s="14" t="inlineStr"/>
-      <c r="AB527" s="14" t="inlineStr"/>
-      <c r="AC527" s="14" t="inlineStr"/>
-      <c r="AD527" s="14" t="inlineStr"/>
+      <c r="AA527" s="14" t="n">
+        <v>1.6721</v>
+      </c>
+      <c r="AB527" s="14" t="n">
+        <v>1.9061</v>
+      </c>
+      <c r="AC527" s="14" t="n">
+        <v>1.8233</v>
+      </c>
+      <c r="AD527" s="14" t="n">
+        <v>1.0107</v>
+      </c>
       <c r="AE527" s="14" t="inlineStr"/>
       <c r="AF527" s="14" t="inlineStr"/>
       <c r="AG527" s="14" t="inlineStr"/>
@@ -68453,15 +68555,27 @@
       <c r="U528" s="14" t="n">
         <v>0.76</v>
       </c>
-      <c r="V528" s="14" t="inlineStr"/>
-      <c r="W528" s="14" t="inlineStr"/>
+      <c r="V528" s="14" t="n">
+        <v>0.8072</v>
+      </c>
+      <c r="W528" s="14" t="n">
+        <v>0.8181</v>
+      </c>
       <c r="X528" s="14" t="inlineStr"/>
       <c r="Y528" s="14" t="inlineStr"/>
       <c r="Z528" s="14" t="inlineStr"/>
-      <c r="AA528" s="14" t="inlineStr"/>
-      <c r="AB528" s="14" t="inlineStr"/>
-      <c r="AC528" s="14" t="inlineStr"/>
-      <c r="AD528" s="14" t="inlineStr"/>
+      <c r="AA528" s="14" t="n">
+        <v>1.7304</v>
+      </c>
+      <c r="AB528" s="14" t="n">
+        <v>2.1437</v>
+      </c>
+      <c r="AC528" s="14" t="n">
+        <v>2.0553</v>
+      </c>
+      <c r="AD528" s="14" t="n">
+        <v>0.9308999999999999</v>
+      </c>
       <c r="AE528" s="14" t="inlineStr"/>
       <c r="AF528" s="14" t="inlineStr"/>
       <c r="AG528" s="14" t="inlineStr"/>
@@ -68599,15 +68713,27 @@
       <c r="U529" s="14" t="n">
         <v>0.47</v>
       </c>
-      <c r="V529" s="14" t="inlineStr"/>
-      <c r="W529" s="14" t="inlineStr"/>
+      <c r="V529" s="14" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="W529" s="14" t="n">
+        <v>0.8435</v>
+      </c>
       <c r="X529" s="14" t="inlineStr"/>
       <c r="Y529" s="14" t="inlineStr"/>
       <c r="Z529" s="14" t="inlineStr"/>
-      <c r="AA529" s="14" t="inlineStr"/>
-      <c r="AB529" s="14" t="inlineStr"/>
-      <c r="AC529" s="14" t="inlineStr"/>
-      <c r="AD529" s="14" t="inlineStr"/>
+      <c r="AA529" s="14" t="n">
+        <v>1.7804</v>
+      </c>
+      <c r="AB529" s="14" t="n">
+        <v>2.1046</v>
+      </c>
+      <c r="AC529" s="14" t="n">
+        <v>2.0562</v>
+      </c>
+      <c r="AD529" s="14" t="n">
+        <v>0.8895999999999999</v>
+      </c>
       <c r="AE529" s="14" t="inlineStr"/>
       <c r="AF529" s="14" t="inlineStr"/>
       <c r="AG529" s="14" t="inlineStr"/>
@@ -68745,15 +68871,27 @@
       <c r="U530" s="14" t="n">
         <v>1.65</v>
       </c>
-      <c r="V530" s="14" t="inlineStr"/>
-      <c r="W530" s="14" t="inlineStr"/>
+      <c r="V530" s="14" t="n">
+        <v>0.8273</v>
+      </c>
+      <c r="W530" s="14" t="n">
+        <v>0.8268</v>
+      </c>
       <c r="X530" s="14" t="inlineStr"/>
       <c r="Y530" s="14" t="inlineStr"/>
       <c r="Z530" s="14" t="inlineStr"/>
-      <c r="AA530" s="14" t="inlineStr"/>
-      <c r="AB530" s="14" t="inlineStr"/>
-      <c r="AC530" s="14" t="inlineStr"/>
-      <c r="AD530" s="14" t="inlineStr"/>
+      <c r="AA530" s="14" t="n">
+        <v>1.7222</v>
+      </c>
+      <c r="AB530" s="14" t="n">
+        <v>2.0817</v>
+      </c>
+      <c r="AC530" s="14" t="n">
+        <v>2.0684</v>
+      </c>
+      <c r="AD530" s="14" t="n">
+        <v>0.9019</v>
+      </c>
       <c r="AE530" s="14" t="inlineStr"/>
       <c r="AF530" s="14" t="inlineStr"/>
       <c r="AG530" s="14" t="inlineStr"/>
@@ -68891,15 +69029,27 @@
       <c r="U531" s="14" t="n">
         <v>0.62</v>
       </c>
-      <c r="V531" s="14" t="inlineStr"/>
-      <c r="W531" s="14" t="inlineStr"/>
+      <c r="V531" s="14" t="n">
+        <v>0.7277</v>
+      </c>
+      <c r="W531" s="14" t="n">
+        <v>0.8003</v>
+      </c>
       <c r="X531" s="14" t="inlineStr"/>
       <c r="Y531" s="14" t="inlineStr"/>
       <c r="Z531" s="14" t="inlineStr"/>
-      <c r="AA531" s="14" t="inlineStr"/>
-      <c r="AB531" s="14" t="inlineStr"/>
-      <c r="AC531" s="14" t="inlineStr"/>
-      <c r="AD531" s="14" t="inlineStr"/>
+      <c r="AA531" s="14" t="n">
+        <v>1.5608</v>
+      </c>
+      <c r="AB531" s="14" t="n">
+        <v>2.1447</v>
+      </c>
+      <c r="AC531" s="14" t="n">
+        <v>2.059</v>
+      </c>
+      <c r="AD531" s="14" t="n">
+        <v>0.8656</v>
+      </c>
       <c r="AE531" s="14" t="inlineStr"/>
       <c r="AF531" s="14" t="inlineStr"/>
       <c r="AG531" s="14" t="inlineStr"/>
@@ -69037,15 +69187,27 @@
       <c r="U532" s="14" t="n">
         <v>0.78</v>
       </c>
-      <c r="V532" s="14" t="inlineStr"/>
-      <c r="W532" s="14" t="inlineStr"/>
+      <c r="V532" s="14" t="n">
+        <v>0.7919</v>
+      </c>
+      <c r="W532" s="14" t="n">
+        <v>0.7823</v>
+      </c>
       <c r="X532" s="14" t="inlineStr"/>
       <c r="Y532" s="14" t="inlineStr"/>
       <c r="Z532" s="14" t="inlineStr"/>
-      <c r="AA532" s="14" t="inlineStr"/>
-      <c r="AB532" s="14" t="inlineStr"/>
-      <c r="AC532" s="14" t="inlineStr"/>
-      <c r="AD532" s="14" t="inlineStr"/>
+      <c r="AA532" s="14" t="n">
+        <v>1.7038</v>
+      </c>
+      <c r="AB532" s="14" t="n">
+        <v>2.1516</v>
+      </c>
+      <c r="AC532" s="14" t="n">
+        <v>2.1172</v>
+      </c>
+      <c r="AD532" s="14" t="n">
+        <v>1.0385</v>
+      </c>
       <c r="AE532" s="14" t="inlineStr"/>
       <c r="AF532" s="14" t="inlineStr"/>
       <c r="AG532" s="14" t="inlineStr"/>
@@ -69183,15 +69345,27 @@
       <c r="U533" s="14" t="n">
         <v>0.61</v>
       </c>
-      <c r="V533" s="14" t="inlineStr"/>
-      <c r="W533" s="14" t="inlineStr"/>
+      <c r="V533" s="14" t="n">
+        <v>0.8254</v>
+      </c>
+      <c r="W533" s="14" t="n">
+        <v>0.7817</v>
+      </c>
       <c r="X533" s="14" t="inlineStr"/>
       <c r="Y533" s="14" t="inlineStr"/>
       <c r="Z533" s="14" t="inlineStr"/>
-      <c r="AA533" s="14" t="inlineStr"/>
-      <c r="AB533" s="14" t="inlineStr"/>
-      <c r="AC533" s="14" t="inlineStr"/>
-      <c r="AD533" s="14" t="inlineStr"/>
+      <c r="AA533" s="14" t="n">
+        <v>1.666</v>
+      </c>
+      <c r="AB533" s="14" t="n">
+        <v>2.0184</v>
+      </c>
+      <c r="AC533" s="14" t="n">
+        <v>1.9403</v>
+      </c>
+      <c r="AD533" s="14" t="n">
+        <v>0.8356</v>
+      </c>
       <c r="AE533" s="14" t="inlineStr"/>
       <c r="AF533" s="14" t="inlineStr"/>
       <c r="AG533" s="14" t="inlineStr"/>
@@ -69329,15 +69503,27 @@
       <c r="U534" s="14" t="n">
         <v>0.76</v>
       </c>
-      <c r="V534" s="14" t="inlineStr"/>
-      <c r="W534" s="14" t="inlineStr"/>
+      <c r="V534" s="14" t="n">
+        <v>0.8375</v>
+      </c>
+      <c r="W534" s="14" t="n">
+        <v>0.8183</v>
+      </c>
       <c r="X534" s="14" t="inlineStr"/>
       <c r="Y534" s="14" t="inlineStr"/>
       <c r="Z534" s="14" t="inlineStr"/>
-      <c r="AA534" s="14" t="inlineStr"/>
-      <c r="AB534" s="14" t="inlineStr"/>
-      <c r="AC534" s="14" t="inlineStr"/>
-      <c r="AD534" s="14" t="inlineStr"/>
+      <c r="AA534" s="14" t="n">
+        <v>1.7724</v>
+      </c>
+      <c r="AB534" s="14" t="n">
+        <v>2.1162</v>
+      </c>
+      <c r="AC534" s="14" t="n">
+        <v>2.076</v>
+      </c>
+      <c r="AD534" s="14" t="n">
+        <v>1.0491</v>
+      </c>
       <c r="AE534" s="14" t="inlineStr"/>
       <c r="AF534" s="14" t="inlineStr"/>
       <c r="AG534" s="14" t="inlineStr"/>
@@ -69475,15 +69661,27 @@
       <c r="U535" s="14" t="n">
         <v>1.58</v>
       </c>
-      <c r="V535" s="14" t="inlineStr"/>
-      <c r="W535" s="14" t="inlineStr"/>
+      <c r="V535" s="14" t="n">
+        <v>0.9481000000000001</v>
+      </c>
+      <c r="W535" s="14" t="n">
+        <v>0.8703</v>
+      </c>
       <c r="X535" s="14" t="inlineStr"/>
       <c r="Y535" s="14" t="inlineStr"/>
       <c r="Z535" s="14" t="inlineStr"/>
-      <c r="AA535" s="14" t="inlineStr"/>
-      <c r="AB535" s="14" t="inlineStr"/>
-      <c r="AC535" s="14" t="inlineStr"/>
-      <c r="AD535" s="14" t="inlineStr"/>
+      <c r="AA535" s="14" t="n">
+        <v>1.8347</v>
+      </c>
+      <c r="AB535" s="14" t="n">
+        <v>1.9351</v>
+      </c>
+      <c r="AC535" s="14" t="n">
+        <v>1.9771</v>
+      </c>
+      <c r="AD535" s="14" t="n">
+        <v>0.7827</v>
+      </c>
       <c r="AE535" s="14" t="inlineStr"/>
       <c r="AF535" s="14" t="inlineStr"/>
       <c r="AG535" s="14" t="inlineStr"/>
@@ -69621,15 +69819,27 @@
       <c r="U536" s="14" t="n">
         <v>1.35</v>
       </c>
-      <c r="V536" s="14" t="inlineStr"/>
-      <c r="W536" s="14" t="inlineStr"/>
+      <c r="V536" s="14" t="n">
+        <v>0.9103</v>
+      </c>
+      <c r="W536" s="14" t="n">
+        <v>0.8986</v>
+      </c>
       <c r="X536" s="14" t="inlineStr"/>
       <c r="Y536" s="14" t="inlineStr"/>
       <c r="Z536" s="14" t="inlineStr"/>
-      <c r="AA536" s="14" t="inlineStr"/>
-      <c r="AB536" s="14" t="inlineStr"/>
-      <c r="AC536" s="14" t="inlineStr"/>
-      <c r="AD536" s="14" t="inlineStr"/>
+      <c r="AA536" s="14" t="n">
+        <v>1.8516</v>
+      </c>
+      <c r="AB536" s="14" t="n">
+        <v>2.034</v>
+      </c>
+      <c r="AC536" s="14" t="n">
+        <v>1.9612</v>
+      </c>
+      <c r="AD536" s="14" t="n">
+        <v>0.8191000000000001</v>
+      </c>
       <c r="AE536" s="14" t="inlineStr"/>
       <c r="AF536" s="14" t="inlineStr"/>
       <c r="AG536" s="14" t="inlineStr"/>
@@ -69767,15 +69977,27 @@
       <c r="U537" s="14" t="n">
         <v>1.31</v>
       </c>
-      <c r="V537" s="14" t="inlineStr"/>
-      <c r="W537" s="14" t="inlineStr"/>
+      <c r="V537" s="14" t="n">
+        <v>0.9124</v>
+      </c>
+      <c r="W537" s="14" t="n">
+        <v>0.9236</v>
+      </c>
       <c r="X537" s="14" t="inlineStr"/>
       <c r="Y537" s="14" t="inlineStr"/>
       <c r="Z537" s="14" t="inlineStr"/>
-      <c r="AA537" s="14" t="inlineStr"/>
-      <c r="AB537" s="14" t="inlineStr"/>
-      <c r="AC537" s="14" t="inlineStr"/>
-      <c r="AD537" s="14" t="inlineStr"/>
+      <c r="AA537" s="14" t="n">
+        <v>1.8977</v>
+      </c>
+      <c r="AB537" s="14" t="n">
+        <v>2.0798</v>
+      </c>
+      <c r="AC537" s="14" t="n">
+        <v>2.003</v>
+      </c>
+      <c r="AD537" s="14" t="n">
+        <v>0.8544</v>
+      </c>
       <c r="AE537" s="14" t="inlineStr"/>
       <c r="AF537" s="14" t="inlineStr"/>
       <c r="AG537" s="14" t="inlineStr"/>
@@ -69913,15 +70135,27 @@
       <c r="U538" s="14" t="n">
         <v>0.98</v>
       </c>
-      <c r="V538" s="14" t="inlineStr"/>
-      <c r="W538" s="14" t="inlineStr"/>
+      <c r="V538" s="14" t="n">
+        <v>0.831</v>
+      </c>
+      <c r="W538" s="14" t="n">
+        <v>0.8846000000000001</v>
+      </c>
       <c r="X538" s="14" t="inlineStr"/>
       <c r="Y538" s="14" t="inlineStr"/>
       <c r="Z538" s="14" t="inlineStr"/>
-      <c r="AA538" s="14" t="inlineStr"/>
-      <c r="AB538" s="14" t="inlineStr"/>
-      <c r="AC538" s="14" t="inlineStr"/>
-      <c r="AD538" s="14" t="inlineStr"/>
+      <c r="AA538" s="14" t="n">
+        <v>1.8375</v>
+      </c>
+      <c r="AB538" s="14" t="n">
+        <v>2.2113</v>
+      </c>
+      <c r="AC538" s="14" t="n">
+        <v>2.3091</v>
+      </c>
+      <c r="AD538" s="14" t="n">
+        <v>1.0362</v>
+      </c>
       <c r="AE538" s="14" t="inlineStr"/>
       <c r="AF538" s="14" t="inlineStr"/>
       <c r="AG538" s="14" t="inlineStr"/>
@@ -70063,15 +70297,27 @@
       <c r="U539" s="14" t="n">
         <v>2.36</v>
       </c>
-      <c r="V539" s="14" t="inlineStr"/>
-      <c r="W539" s="14" t="inlineStr"/>
+      <c r="V539" s="14" t="n">
+        <v>0.9036999999999999</v>
+      </c>
+      <c r="W539" s="14" t="n">
+        <v>0.8824</v>
+      </c>
       <c r="X539" s="14" t="inlineStr"/>
       <c r="Y539" s="14" t="inlineStr"/>
       <c r="Z539" s="14" t="inlineStr"/>
-      <c r="AA539" s="14" t="inlineStr"/>
-      <c r="AB539" s="14" t="inlineStr"/>
-      <c r="AC539" s="14" t="inlineStr"/>
-      <c r="AD539" s="14" t="inlineStr"/>
+      <c r="AA539" s="14" t="n">
+        <v>1.9363</v>
+      </c>
+      <c r="AB539" s="14" t="n">
+        <v>2.1427</v>
+      </c>
+      <c r="AC539" s="14" t="n">
+        <v>2.2092</v>
+      </c>
+      <c r="AD539" s="14" t="n">
+        <v>0.8803</v>
+      </c>
       <c r="AE539" s="14" t="inlineStr"/>
       <c r="AF539" s="14" t="inlineStr"/>
       <c r="AG539" s="14" t="inlineStr"/>
@@ -70209,15 +70455,27 @@
       <c r="U540" s="14" t="n">
         <v>5.77</v>
       </c>
-      <c r="V540" s="14" t="inlineStr"/>
-      <c r="W540" s="14" t="inlineStr"/>
+      <c r="V540" s="14" t="n">
+        <v>0.7133</v>
+      </c>
+      <c r="W540" s="14" t="n">
+        <v>0.8159999999999999</v>
+      </c>
       <c r="X540" s="14" t="inlineStr"/>
       <c r="Y540" s="14" t="inlineStr"/>
       <c r="Z540" s="14" t="inlineStr"/>
-      <c r="AA540" s="14" t="inlineStr"/>
-      <c r="AB540" s="14" t="inlineStr"/>
-      <c r="AC540" s="14" t="inlineStr"/>
-      <c r="AD540" s="14" t="inlineStr"/>
+      <c r="AA540" s="14" t="n">
+        <v>1.6883</v>
+      </c>
+      <c r="AB540" s="14" t="n">
+        <v>2.367</v>
+      </c>
+      <c r="AC540" s="14" t="n">
+        <v>2.3625</v>
+      </c>
+      <c r="AD540" s="14" t="n">
+        <v>0.828</v>
+      </c>
       <c r="AE540" s="14" t="inlineStr"/>
       <c r="AF540" s="14" t="inlineStr"/>
       <c r="AG540" s="14" t="inlineStr"/>
@@ -70355,15 +70613,27 @@
       <c r="U541" s="14" t="n">
         <v>4.39</v>
       </c>
-      <c r="V541" s="14" t="inlineStr"/>
-      <c r="W541" s="14" t="inlineStr"/>
+      <c r="V541" s="14" t="n">
+        <v>1.1058</v>
+      </c>
+      <c r="W541" s="14" t="n">
+        <v>0.9076</v>
+      </c>
       <c r="X541" s="14" t="inlineStr"/>
       <c r="Y541" s="14" t="inlineStr"/>
       <c r="Z541" s="14" t="inlineStr"/>
-      <c r="AA541" s="14" t="inlineStr"/>
-      <c r="AB541" s="14" t="inlineStr"/>
-      <c r="AC541" s="14" t="inlineStr"/>
-      <c r="AD541" s="14" t="inlineStr"/>
+      <c r="AA541" s="14" t="n">
+        <v>2.2381</v>
+      </c>
+      <c r="AB541" s="14" t="n">
+        <v>2.0239</v>
+      </c>
+      <c r="AC541" s="14" t="n">
+        <v>1.8114</v>
+      </c>
+      <c r="AD541" s="14" t="n">
+        <v>0.8546</v>
+      </c>
       <c r="AE541" s="14" t="inlineStr"/>
       <c r="AF541" s="14" t="inlineStr"/>
       <c r="AG541" s="14" t="inlineStr"/>
@@ -70501,15 +70771,27 @@
       <c r="U542" s="14" t="n">
         <v>1.23</v>
       </c>
-      <c r="V542" s="14" t="inlineStr"/>
-      <c r="W542" s="14" t="inlineStr"/>
+      <c r="V542" s="14" t="n">
+        <v>1.0515</v>
+      </c>
+      <c r="W542" s="14" t="n">
+        <v>0.9569</v>
+      </c>
       <c r="X542" s="14" t="inlineStr"/>
       <c r="Y542" s="14" t="inlineStr"/>
       <c r="Z542" s="14" t="inlineStr"/>
-      <c r="AA542" s="14" t="inlineStr"/>
-      <c r="AB542" s="14" t="inlineStr"/>
-      <c r="AC542" s="14" t="inlineStr"/>
-      <c r="AD542" s="14" t="inlineStr"/>
+      <c r="AA542" s="14" t="n">
+        <v>2.2345</v>
+      </c>
+      <c r="AB542" s="14" t="n">
+        <v>2.125</v>
+      </c>
+      <c r="AC542" s="14" t="n">
+        <v>1.8555</v>
+      </c>
+      <c r="AD542" s="14" t="n">
+        <v>0.9241</v>
+      </c>
       <c r="AE542" s="14" t="inlineStr"/>
       <c r="AF542" s="14" t="inlineStr"/>
       <c r="AG542" s="14" t="inlineStr"/>
@@ -70647,15 +70929,27 @@
       <c r="U543" s="14" t="n">
         <v>1.35</v>
       </c>
-      <c r="V543" s="14" t="inlineStr"/>
-      <c r="W543" s="14" t="inlineStr"/>
+      <c r="V543" s="14" t="n">
+        <v>1.121</v>
+      </c>
+      <c r="W543" s="14" t="n">
+        <v>1.0928</v>
+      </c>
       <c r="X543" s="14" t="inlineStr"/>
       <c r="Y543" s="14" t="inlineStr"/>
       <c r="Z543" s="14" t="inlineStr"/>
-      <c r="AA543" s="14" t="inlineStr"/>
-      <c r="AB543" s="14" t="inlineStr"/>
-      <c r="AC543" s="14" t="inlineStr"/>
-      <c r="AD543" s="14" t="inlineStr"/>
+      <c r="AA543" s="14" t="n">
+        <v>2.2404</v>
+      </c>
+      <c r="AB543" s="14" t="n">
+        <v>1.9985</v>
+      </c>
+      <c r="AC543" s="14" t="n">
+        <v>1.7747</v>
+      </c>
+      <c r="AD543" s="14" t="n">
+        <v>0.8663</v>
+      </c>
       <c r="AE543" s="14" t="inlineStr"/>
       <c r="AF543" s="14" t="inlineStr"/>
       <c r="AG543" s="14" t="inlineStr"/>
@@ -70793,15 +71087,27 @@
       <c r="U544" s="14" t="n">
         <v>2.23</v>
       </c>
-      <c r="V544" s="14" t="inlineStr"/>
-      <c r="W544" s="14" t="inlineStr"/>
+      <c r="V544" s="14" t="n">
+        <v>1.1948</v>
+      </c>
+      <c r="W544" s="14" t="n">
+        <v>1.1224</v>
+      </c>
       <c r="X544" s="14" t="inlineStr"/>
       <c r="Y544" s="14" t="inlineStr"/>
       <c r="Z544" s="14" t="inlineStr"/>
-      <c r="AA544" s="14" t="inlineStr"/>
-      <c r="AB544" s="14" t="inlineStr"/>
-      <c r="AC544" s="14" t="inlineStr"/>
-      <c r="AD544" s="14" t="inlineStr"/>
+      <c r="AA544" s="14" t="n">
+        <v>2.4095</v>
+      </c>
+      <c r="AB544" s="14" t="n">
+        <v>2.0166</v>
+      </c>
+      <c r="AC544" s="14" t="n">
+        <v>1.7663</v>
+      </c>
+      <c r="AD544" s="14" t="n">
+        <v>0.6137</v>
+      </c>
       <c r="AE544" s="14" t="inlineStr"/>
       <c r="AF544" s="14" t="inlineStr"/>
       <c r="AG544" s="14" t="inlineStr"/>
@@ -70939,15 +71245,27 @@
       <c r="U545" s="14" t="n">
         <v>2.85</v>
       </c>
-      <c r="V545" s="14" t="inlineStr"/>
-      <c r="W545" s="14" t="inlineStr"/>
+      <c r="V545" s="14" t="n">
+        <v>1.9668</v>
+      </c>
+      <c r="W545" s="14" t="n">
+        <v>1.4275</v>
+      </c>
       <c r="X545" s="14" t="inlineStr"/>
       <c r="Y545" s="14" t="inlineStr"/>
       <c r="Z545" s="14" t="inlineStr"/>
-      <c r="AA545" s="14" t="inlineStr"/>
-      <c r="AB545" s="14" t="inlineStr"/>
-      <c r="AC545" s="14" t="inlineStr"/>
-      <c r="AD545" s="14" t="inlineStr"/>
+      <c r="AA545" s="14" t="n">
+        <v>4.4272</v>
+      </c>
+      <c r="AB545" s="14" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="AC545" s="14" t="n">
+        <v>1.7624</v>
+      </c>
+      <c r="AD545" s="14" t="n">
+        <v>0.7639</v>
+      </c>
       <c r="AE545" s="14" t="inlineStr"/>
       <c r="AF545" s="14" t="inlineStr"/>
       <c r="AG545" s="14" t="inlineStr"/>
@@ -71085,15 +71403,27 @@
       <c r="U546" s="14" t="n">
         <v>3.07</v>
       </c>
-      <c r="V546" s="14" t="inlineStr"/>
-      <c r="W546" s="14" t="inlineStr"/>
+      <c r="V546" s="14" t="n">
+        <v>1.6302</v>
+      </c>
+      <c r="W546" s="14" t="n">
+        <v>1.5973</v>
+      </c>
       <c r="X546" s="14" t="inlineStr"/>
       <c r="Y546" s="14" t="inlineStr"/>
       <c r="Z546" s="14" t="inlineStr"/>
-      <c r="AA546" s="14" t="inlineStr"/>
-      <c r="AB546" s="14" t="inlineStr"/>
-      <c r="AC546" s="14" t="inlineStr"/>
-      <c r="AD546" s="14" t="inlineStr"/>
+      <c r="AA546" s="14" t="n">
+        <v>5.1115</v>
+      </c>
+      <c r="AB546" s="14" t="n">
+        <v>3.1356</v>
+      </c>
+      <c r="AC546" s="14" t="n">
+        <v>2.3557</v>
+      </c>
+      <c r="AD546" s="14" t="n">
+        <v>0.9451000000000001</v>
+      </c>
       <c r="AE546" s="14" t="inlineStr"/>
       <c r="AF546" s="14" t="inlineStr"/>
       <c r="AG546" s="14" t="inlineStr"/>
@@ -71231,15 +71561,27 @@
       <c r="U547" s="14" t="n">
         <v>27.02</v>
       </c>
-      <c r="V547" s="14" t="inlineStr"/>
-      <c r="W547" s="14" t="inlineStr"/>
+      <c r="V547" s="14" t="n">
+        <v>1.7373</v>
+      </c>
+      <c r="W547" s="14" t="n">
+        <v>1.7781</v>
+      </c>
       <c r="X547" s="14" t="inlineStr"/>
       <c r="Y547" s="14" t="inlineStr"/>
       <c r="Z547" s="14" t="inlineStr"/>
-      <c r="AA547" s="14" t="inlineStr"/>
-      <c r="AB547" s="14" t="inlineStr"/>
-      <c r="AC547" s="14" t="inlineStr"/>
-      <c r="AD547" s="14" t="inlineStr"/>
+      <c r="AA547" s="14" t="n">
+        <v>5.3391</v>
+      </c>
+      <c r="AB547" s="14" t="n">
+        <v>3.0733</v>
+      </c>
+      <c r="AC547" s="14" t="n">
+        <v>2.3591</v>
+      </c>
+      <c r="AD547" s="14" t="n">
+        <v>0.9615</v>
+      </c>
       <c r="AE547" s="14" t="inlineStr"/>
       <c r="AF547" s="14" t="inlineStr"/>
       <c r="AG547" s="14" t="inlineStr"/>

</xml_diff>